<commit_message>
Fix indirect-export dates not parsing (DD-MM-YYYY): $553K now in yearly KPI/trend
- parse_date: add %d-%m-%Y (and %Y/%m/%d) — PDF invoice dates like 03-07-2026 were
  returning None -> yil=0 -> indirect revenue excluded from trend/KPI but present in
  customer/product/country totals ($6.58M vs $7.13M mismatch)
- Now consistent: total $7.13M; indirect adds 2023 +$35K/2024 +$139K/2025 +$321K/2026 +$59K
- Add MUSTERI_LISTESI.xlsx (90 customers)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoehW9ESGDK2XkibhR7KNP
</commit_message>
<xml_diff>
--- a/data/MUSTERI_LISTESI.xlsx
+++ b/data/MUSTERI_LISTESI.xlsx
@@ -1046,10 +1046,18 @@
       <c r="H13" t="n">
         <v>11112</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2024-10-04</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
       <c r="K13" t="n">
-        <v>9999</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14">
@@ -1508,10 +1516,18 @@
       <c r="H23" t="n">
         <v>20685</v>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2025-03-02</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
       <c r="K23" t="n">
-        <v>9999</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24">
@@ -1688,10 +1704,18 @@
       <c r="H27" t="n">
         <v>28493</v>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2025-06-18</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
       <c r="K27" t="n">
-        <v>9999</v>
+        <v>245</v>
       </c>
     </row>
     <row r="28">
@@ -1821,10 +1845,18 @@
       <c r="H30" t="n">
         <v>7495</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2023-10-01</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
       <c r="K30" t="n">
-        <v>9999</v>
+        <v>305</v>
       </c>
     </row>
     <row r="31">
@@ -2800,10 +2832,18 @@
       <c r="H51" t="n">
         <v>28441</v>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
       <c r="K51" t="n">
-        <v>9999</v>
+        <v>438</v>
       </c>
     </row>
     <row r="52">
@@ -2886,10 +2926,18 @@
       <c r="H53" t="n">
         <v>12076</v>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2025-04-08</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="K53" t="n">
-        <v>9999</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54">
@@ -3066,10 +3114,18 @@
       <c r="H57" t="n">
         <v>8703</v>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2023-10-24</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2024-02-23</t>
+        </is>
+      </c>
       <c r="K57" t="n">
-        <v>9999</v>
+        <v>913</v>
       </c>
     </row>
     <row r="58">
@@ -3293,10 +3349,18 @@
       <c r="H62" t="n">
         <v>3624</v>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2024-11-04</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
       <c r="K62" t="n">
-        <v>9999</v>
+        <v>52</v>
       </c>
     </row>
     <row r="63">
@@ -3520,10 +3584,18 @@
       <c r="H67" t="n">
         <v>9000</v>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="K67" t="n">
-        <v>9999</v>
+        <v>94</v>
       </c>
     </row>
     <row r="68">
@@ -3747,10 +3819,18 @@
       <c r="H72" t="n">
         <v>2388</v>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2024-01-05</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2024-05-13</t>
+        </is>
+      </c>
       <c r="K72" t="n">
-        <v>9999</v>
+        <v>833</v>
       </c>
     </row>
     <row r="73">
@@ -3974,10 +4054,18 @@
       <c r="H77" t="n">
         <v>6083</v>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2024-12-04</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>2024-12-04</t>
+        </is>
+      </c>
       <c r="K77" t="n">
-        <v>9999</v>
+        <v>628</v>
       </c>
     </row>
     <row r="78">
@@ -4248,10 +4336,18 @@
       <c r="H83" t="n">
         <v>3689</v>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2023-10-17</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>2023-10-17</t>
+        </is>
+      </c>
       <c r="K83" t="n">
-        <v>9999</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="84">
@@ -4287,10 +4383,18 @@
       <c r="H84" t="n">
         <v>1500</v>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2025-07-21</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2025-07-21</t>
+        </is>
+      </c>
       <c r="K84" t="n">
-        <v>9999</v>
+        <v>399</v>
       </c>
     </row>
     <row r="85">
@@ -4326,10 +4430,18 @@
       <c r="H85" t="n">
         <v>1479</v>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2025-03-11</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>2025-03-11</t>
+        </is>
+      </c>
       <c r="K85" t="n">
-        <v>9999</v>
+        <v>531</v>
       </c>
     </row>
     <row r="86">
@@ -4459,10 +4571,18 @@
       <c r="H88" t="n">
         <v>1053</v>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2024-12-23</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2024-12-23</t>
+        </is>
+      </c>
       <c r="K88" t="n">
-        <v>9999</v>
+        <v>609</v>
       </c>
     </row>
     <row r="89">
@@ -4498,10 +4618,18 @@
       <c r="H89" t="n">
         <v>588</v>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2025-03-14</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>2025-03-14</t>
+        </is>
+      </c>
       <c r="K89" t="n">
-        <v>9999</v>
+        <v>528</v>
       </c>
     </row>
     <row r="90">
@@ -4584,10 +4712,18 @@
       <c r="H91" t="n">
         <v>499</v>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2024-01-03</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>2024-01-03</t>
+        </is>
+      </c>
       <c r="K91" t="n">
-        <v>9999</v>
+        <v>964</v>
       </c>
     </row>
     <row r="93">

</xml_diff>